<commit_message>
auto sync 2026-09-29 07:28 KST
</commit_message>
<xml_diff>
--- a/봉제현황/일별이미지/일별이미지_누적.xlsx
+++ b/봉제현황/일별이미지/일별이미지_누적.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M47"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3286,6 +3286,128 @@
         </is>
       </c>
       <c r="M47" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:40</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>new-01.png</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-09-28/new-01.png</t>
+        </is>
+      </c>
+      <c r="F48" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>1082823</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:40</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>본문날짜칸공란→파일명9/28 애리후세540(460+80)</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>2026-09-28_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>667c63a245be75f43dd2d4f70e45cf456b39b80aec352d224d0ea6f382b800e8</t>
+        </is>
+      </c>
+      <c r="M48" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:40</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>p-01.png</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-09-28/p-01.png</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>1082823</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:40</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>본문날짜칸공란→파일명9/28 애리후세540(460+80)</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>2026-09-28_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>667c63a245be75f43dd2d4f70e45cf456b39b80aec352d224d0ea6f382b800e8</t>
+        </is>
+      </c>
+      <c r="M49" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3301,7 +3423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3477,6 +3599,73 @@
       <c r="H5" t="inlineStr">
         <is>
           <t>2026-09-21 18:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-09-28_일지.pdf</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>667c63a245be75f43dd2d4f70e45cf456b39b80aec352d224d0ea6f382b800e8</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>636727</v>
+      </c>
+      <c r="D6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>본문날짜칸공란→파일명9/28 애리후세540(460+80)</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>봉제생산현황_묶음.pdf</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>89a489512ab370bfc9ff60fe880c196f44d9f5049c8848ed859bc2887244a780</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>32587011</v>
+      </c>
+      <c r="D7" t="n">
+        <v>46</v>
+      </c>
+      <c r="E7" t="n">
+        <v>46</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>9/28 1p append(45→46)</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto sync 2026-10-01 09:04 KST
</commit_message>
<xml_diff>
--- a/봉제현황/일별이미지/일별이미지_누적.xlsx
+++ b/봉제현황/일별이미지/일별이미지_누적.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3408,6 +3408,250 @@
         </is>
       </c>
       <c r="M49" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:10</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>new-01.png</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-09-29/new-01.png</t>
+        </is>
+      </c>
+      <c r="F50" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>1096164</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:10</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>본문09/29확정 애리후세582</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>2026-09-29_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>4e7a0856520d01f7e9d097de660cdbb9a47966731c8cd16fd65868d35f99c05e</t>
+        </is>
+      </c>
+      <c r="M50" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:10</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>p-01.png</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-09-29/p-01.png</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>1096164</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:10</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>본문09/29확정 애리후세582</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>2026-09-29_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>4e7a0856520d01f7e9d097de660cdbb9a47966731c8cd16fd65868d35f99c05e</t>
+        </is>
+      </c>
+      <c r="M51" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:10</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>new-01.png</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-09-30/new-01.png</t>
+        </is>
+      </c>
+      <c r="F52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>1049300</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:10</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>본문09/30확정 애리후세683</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>2026-09-30_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>3e02742a148b57ebd0f610470daa709f838c56585b72384cb51dcd8d0682d316</t>
+        </is>
+      </c>
+      <c r="M52" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:10</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>p-01.png</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-09-30/p-01.png</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="H53" t="n">
+        <v>1049300</v>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:10</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>본문09/30확정 애리후세683</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>2026-09-30_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>3e02742a148b57ebd0f610470daa709f838c56585b72384cb51dcd8d0682d316</t>
+        </is>
+      </c>
+      <c r="M53" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3423,7 +3667,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3666,6 +3910,109 @@
       <c r="H7" t="inlineStr">
         <is>
           <t>2026-09-28 19:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-09-29_일지.pdf</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>4e7a0856520d01f7e9d097de660cdbb9a47966731c8cd16fd65868d35f99c05e</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>636375</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>본문09/29확정 애리후세582</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-09-30_일지.pdf</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>3e02742a148b57ebd0f610470daa709f838c56585b72384cb51dcd8d0682d316</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>626255</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>본문09/30확정 애리후세683</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>봉제생산현황_묶음.pdf</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>169b25f3480f71d94e19b27226a63281c96083eea3a667fd2faca107fcd41a56</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>33840867</v>
+      </c>
+      <c r="D10" t="n">
+        <v>48</v>
+      </c>
+      <c r="E10" t="n">
+        <v>48</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>9/29·9/30 2p append(46→48)</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-10-01 09:10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto sync 2026-10-02 08:05 KST
</commit_message>
<xml_diff>
--- a/봉제현황/일별이미지/일별이미지_누적.xlsx
+++ b/봉제현황/일별이미지/일별이미지_누적.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M53"/>
+  <dimension ref="A1:M55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3652,6 +3652,128 @@
         </is>
       </c>
       <c r="M53" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:57</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>new-01.png</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-01/new-01.png</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>1074121</v>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:57</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>본문10/01확정 애리후세607</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>2026-10-01_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>6a80653cd96669e7b39598f9404a8b0f39296f032bed6b0dd4994b051840d23e</t>
+        </is>
+      </c>
+      <c r="M54" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:57</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>p-01.png</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-01/p-01.png</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="H55" t="n">
+        <v>1074121</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:57</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>본문10/01확정 애리후세607</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>2026-10-01_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>6a80653cd96669e7b39598f9404a8b0f39296f032bed6b0dd4994b051840d23e</t>
+        </is>
+      </c>
+      <c r="M55" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3667,7 +3789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4013,6 +4135,73 @@
       <c r="H10" t="inlineStr">
         <is>
           <t>2026-10-01 09:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-01_일지.pdf</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>6a80653cd96669e7b39598f9404a8b0f39296f032bed6b0dd4994b051840d23e</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>633191</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>본문10/01확정 애리후세607</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>봉제생산현황_묶음.pdf</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>e1e15eccdef5ced35d29791509d3ea43a45fbc89608d0354b7246016d414886c</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>34469673</v>
+      </c>
+      <c r="D12" t="n">
+        <v>49</v>
+      </c>
+      <c r="E12" t="n">
+        <v>49</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>10/1 1p append(48→49)</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:57</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto sync 2026-10-06 08:05 KST
</commit_message>
<xml_diff>
--- a/봉제현황/일별이미지/일별이미지_누적.xlsx
+++ b/봉제현황/일별이미지/일별이미지_누적.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M55"/>
+  <dimension ref="A1:M59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3774,6 +3774,250 @@
         </is>
       </c>
       <c r="M55" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:23</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>new-01.png</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-02/new-01.png</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="H56" t="n">
+        <v>1044199</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:23</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>본문10/02확정 애리후세404</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>2026-10-02_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>2523d530f2120d64e0cb251d92a99bed57871d5a1a444ba7a9d7746200cd19f6</t>
+        </is>
+      </c>
+      <c r="M56" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:23</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>p-01.png</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-02/p-01.png</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="H57" t="n">
+        <v>1044199</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:23</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>본문10/02확정 애리후세404</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>2026-10-02_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>2523d530f2120d64e0cb251d92a99bed57871d5a1a444ba7a9d7746200cd19f6</t>
+        </is>
+      </c>
+      <c r="M57" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:23</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>new-01.png</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-03/new-01.png</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="H58" t="n">
+        <v>1015457</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:23</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>본문10/03확정 애리후세323</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>2026-10-03_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>a7c24385777c805435af0858840e124f9d3875260635886050df364cc2eaf4be</t>
+        </is>
+      </c>
+      <c r="M58" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:23</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>p-01.png</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-03/p-01.png</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="H59" t="n">
+        <v>1015457</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:23</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>본문10/03확정 애리후세323</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>2026-10-03_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>a7c24385777c805435af0858840e124f9d3875260635886050df364cc2eaf4be</t>
+        </is>
+      </c>
+      <c r="M59" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3789,7 +4033,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4202,6 +4446,109 @@
       <c r="H12" t="inlineStr">
         <is>
           <t>2026-10-02 07:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-02_일지.pdf</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2523d530f2120d64e0cb251d92a99bed57871d5a1a444ba7a9d7746200cd19f6</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>615583</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>본문10/02확정 애리후세404</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-03_일지.pdf</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>a7c24385777c805435af0858840e124f9d3875260635886050df364cc2eaf4be</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>611471</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-10-03</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>본문10/03확정 애리후세323</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>봉제생산현황_묶음.pdf</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>7bef87e613445d91feb0f0b49c2e3148ae5eaced1524292d3e11280537920fa1</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>35687953</v>
+      </c>
+      <c r="D15" t="n">
+        <v>51</v>
+      </c>
+      <c r="E15" t="n">
+        <v>51</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>10/2·10/3 2p append(49→51)</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-10-06 07:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto sync 2026-10-06 18:05 KST
</commit_message>
<xml_diff>
--- a/봉제현황/일별이미지/일별이미지_누적.xlsx
+++ b/봉제현황/일별이미지/일별이미지_누적.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M59"/>
+  <dimension ref="A1:M61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4018,6 +4018,128 @@
         </is>
       </c>
       <c r="M59" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-10-06 17:54</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>new-01.png</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-06/new-01.png</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="H60" t="n">
+        <v>1031745</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>2026-10-06 17:54</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>본문10/06확정 애리후세240</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>2026-10-06_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>ff7139ba479535643ca9ae914eb763524098b714f1008d41c8f778cb8efd36d7</t>
+        </is>
+      </c>
+      <c r="M60" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-10-06 17:54</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>p-01.png</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-06/p-01.png</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="H61" t="n">
+        <v>1031745</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>2026-10-06 17:54</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>본문10/06확정 애리후세240</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>2026-10-06_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>ff7139ba479535643ca9ae914eb763524098b714f1008d41c8f778cb8efd36d7</t>
+        </is>
+      </c>
+      <c r="M61" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4033,7 +4155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4549,6 +4671,73 @@
       <c r="H15" t="inlineStr">
         <is>
           <t>2026-10-06 07:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-10-06_일지.pdf</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ff7139ba479535643ca9ae914eb763524098b714f1008d41c8f778cb8efd36d7</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>617951</v>
+      </c>
+      <c r="D16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>본문10/06확정 애리후세240</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-10-06 17:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>봉제생산현황_묶음.pdf</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>6e92b797f2e122d1c81d443ebbd335a961c3f8e4ab67790e7eb6abfc18f16ce4</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>36301515</v>
+      </c>
+      <c r="D17" t="n">
+        <v>52</v>
+      </c>
+      <c r="E17" t="n">
+        <v>52</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>10/6 1p append(51→52)</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-10-06 17:54</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto sync 2026-10-07 18:30 KST
</commit_message>
<xml_diff>
--- a/봉제현황/일별이미지/일별이미지_누적.xlsx
+++ b/봉제현황/일별이미지/일별이미지_누적.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M61"/>
+  <dimension ref="A1:M63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4140,6 +4140,128 @@
         </is>
       </c>
       <c r="M61" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-10-07 18:17</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>new-01.png</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-07/new-01.png</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="H62" t="n">
+        <v>1065442</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>2026-10-07 18:17</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>본문10/07확정 애리후세판독보류(240/230)</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>2026-10-07_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>47f037beff7fa8f843bf7c4adcaff297a4cd463abce28d85d69afa0cb49377d3</t>
+        </is>
+      </c>
+      <c r="M62" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-10-07 18:17</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>p-01.png</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-07/p-01.png</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="H63" t="n">
+        <v>1065442</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>2026-10-07 18:17</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>본문10/07확정 애리후세판독보류(240/230)</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>2026-10-07_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>47f037beff7fa8f843bf7c4adcaff297a4cd463abce28d85d69afa0cb49377d3</t>
+        </is>
+      </c>
+      <c r="M63" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4155,7 +4277,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4738,6 +4860,73 @@
       <c r="H17" t="inlineStr">
         <is>
           <t>2026-10-06 17:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-10-07_일지.pdf</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>47f037beff7fa8f843bf7c4adcaff297a4cd463abce28d85d69afa0cb49377d3</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>627583</v>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>본문10/07확정 애리후세판독보류(240/230)</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-10-07 18:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>봉제생산현황_묶음.pdf</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>ea2617d69610a61dc4c0305e454e4db50a6ddbd6cbdd257cd3d20aed19ae442d</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>36924711</v>
+      </c>
+      <c r="D19" t="n">
+        <v>53</v>
+      </c>
+      <c r="E19" t="n">
+        <v>53</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>10/7 1p append(52→53)</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-10-07 18:17</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto sync 2026-10-09 07:24 KST
</commit_message>
<xml_diff>
--- a/봉제현황/일별이미지/일별이미지_누적.xlsx
+++ b/봉제현황/일별이미지/일별이미지_누적.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M64"/>
+  <dimension ref="A1:M66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4323,6 +4323,128 @@
         </is>
       </c>
       <c r="M64" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:18</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>new-01.png</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-08/new-01.png</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="H65" t="n">
+        <v>1070769</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:18</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>본문10/08확정 애리후세430</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>2026-10-08_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>803e09cf9f144b3aac05b969aa0be8d66be4be92339ce880e17c12b68040fdc3</t>
+        </is>
+      </c>
+      <c r="M65" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:18</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>p-01.png</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-08/p-01.png</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="H66" t="n">
+        <v>1070769</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:18</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>본문10/08확정 애리후세430</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>2026-10-08_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>803e09cf9f144b3aac05b969aa0be8d66be4be92339ce880e17c12b68040fdc3</t>
+        </is>
+      </c>
+      <c r="M66" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4338,7 +4460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4988,6 +5110,73 @@
       <c r="H19" t="inlineStr">
         <is>
           <t>2026-10-07 18:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-08_일지.pdf</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>803e09cf9f144b3aac05b969aa0be8d66be4be92339ce880e17c12b68040fdc3</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>629143</v>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>본문10/08확정 애리후세430</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>봉제생산현황_묶음.pdf</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>47a93474f669778b6dac80f86a14143381dfde7ee0cef3b1de0daafa9dbc80b7</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>37546376</v>
+      </c>
+      <c r="D21" t="n">
+        <v>54</v>
+      </c>
+      <c r="E21" t="n">
+        <v>54</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>10/8 1p append(53→54)</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-10-09 07:18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto sync 2026-10-10 07:49 KST
</commit_message>
<xml_diff>
--- a/봉제현황/일별이미지/일별이미지_누적.xlsx
+++ b/봉제현황/일별이미지/일별이미지_누적.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M66"/>
+  <dimension ref="A1:M68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4445,6 +4445,128 @@
         </is>
       </c>
       <c r="M66" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-10-10 07:41</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>new-01.png</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-09/new-01.png</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="H67" t="n">
+        <v>1028475</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>2026-10-10 07:41</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>본문10/09확정 애리후세279</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>2026-10-09_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>07f597b785eb6d1357ad95bc06773d9736064ead51339ffbf3b9c9544a7e782f</t>
+        </is>
+      </c>
+      <c r="M67" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-10-10 07:41</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>p-01.png</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-09/p-01.png</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="H68" t="n">
+        <v>1028475</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>2026-10-10 07:41</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>본문10/09확정 애리후세279</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>2026-10-09_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>07f597b785eb6d1357ad95bc06773d9736064ead51339ffbf3b9c9544a7e782f</t>
+        </is>
+      </c>
+      <c r="M68" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4460,7 +4582,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H21"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5177,6 +5299,73 @@
       <c r="H21" t="inlineStr">
         <is>
           <t>2026-10-09 07:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-09_일지.pdf</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>07f597b785eb6d1357ad95bc06773d9736064ead51339ffbf3b9c9544a7e782f</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>615887</v>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>2026-10-09</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>본문10/09확정 애리후세279</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-10-10 07:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>봉제생산현황_묶음.pdf</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2de41790c514bbfd706f4a02d5ba334285a46b3e8f69ed2e791c45a3f2c3fbf4</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>38157650</v>
+      </c>
+      <c r="D23" t="n">
+        <v>55</v>
+      </c>
+      <c r="E23" t="n">
+        <v>55</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>10/9 1p append(54→55)</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-10-10 07:41</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto sync 2026-10-16 17:54 KST
</commit_message>
<xml_diff>
--- a/봉제현황/일별이미지/일별이미지_누적.xlsx
+++ b/봉제현황/일별이미지/일별이미지_누적.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="원장" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="PDF처리" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="요약" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="원장보조" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="원장" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PDF처리" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="원장보조" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'원장'!$A$1:$M$43</definedName>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M68"/>
+  <dimension ref="A1:M74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4567,6 +4567,372 @@
         </is>
       </c>
       <c r="M68" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>new-01.png</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-13/new-01.png</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="H69" t="n">
+        <v>975985</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>본문10/13확정 애리후세미기재(칸 비어 있음)</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>2026-10-13_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>574eef056b660be8171513760b85dcafb562be5b7fa3fab35cfed8b8d74cb111</t>
+        </is>
+      </c>
+      <c r="M69" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>p-01.png</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-13/p-01.png</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="H70" t="n">
+        <v>975985</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>본문10/13확정 애리후세미기재(칸 비어 있음)</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>2026-10-13_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>574eef056b660be8171513760b85dcafb562be5b7fa3fab35cfed8b8d74cb111</t>
+        </is>
+      </c>
+      <c r="M70" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>new-01.png</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-14/new-01.png</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="H71" t="n">
+        <v>1093238</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>본문10/14확정 애리후세417</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>2026-10-14_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>09d656aa6d621f0bd3f373a374a2e33430a2d7a9f4f796156abebedcff0ff5bf</t>
+        </is>
+      </c>
+      <c r="M71" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>p-01.png</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-14/p-01.png</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="H72" t="n">
+        <v>1093238</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>본문10/14확정 애리후세417</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>2026-10-14_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>09d656aa6d621f0bd3f373a374a2e33430a2d7a9f4f796156abebedcff0ff5bf</t>
+        </is>
+      </c>
+      <c r="M72" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>new-01.png</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-15/new-01.png</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="H73" t="n">
+        <v>1056435</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>본문10/15확정 애리후세545</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>2026-10-15_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>7e3b15ecfcff3d14861f32351a00d15601c037baca429bf1d9b7f4cf6d34d1b1</t>
+        </is>
+      </c>
+      <c r="M73" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>p-01.png</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>일별이미지/2026-10-15/p-01.png</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>page</t>
+        </is>
+      </c>
+      <c r="H74" t="n">
+        <v>1056435</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>본문10/15확정 애리후세545</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>2026-10-15_일지.pdf</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>7e3b15ecfcff3d14861f32351a00d15601c037baca429bf1d9b7f4cf6d34d1b1</t>
+        </is>
+      </c>
+      <c r="M74" t="b">
         <v>1</v>
       </c>
     </row>
@@ -4582,7 +4948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5366,6 +5732,145 @@
       <c r="H23" t="inlineStr">
         <is>
           <t>2026-10-10 07:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-13_일지.pdf</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>574eef056b660be8171513760b85dcafb562be5b7fa3fab35cfed8b8d74cb111</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>579367</v>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>본문10/13확정 애리후세미기재(칸 비어 있음)</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-14_일지.pdf</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>09d656aa6d621f0bd3f373a374a2e33430a2d7a9f4f796156abebedcff0ff5bf</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>614967</v>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>본문10/14확정 애리후세417</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-15_일지.pdf</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>7e3b15ecfcff3d14861f32351a00d15601c037baca429bf1d9b7f4cf6d34d1b1</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>608807</v>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>본문10/15확정 애리후세545</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>봉제생산현황_묶음.pdf</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>57ab2d96ec4edc827ca667e6faaf73e309c539fb11714cc4d521cb87b257f1e4</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>39946952</v>
+      </c>
+      <c r="D27" t="n">
+        <v>58</v>
+      </c>
+      <c r="E27" t="n">
+        <v>58</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>10/13·10/14·10/15 3p append(55→58)</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2026-10-16 11:53</t>
         </is>
       </c>
     </row>

</xml_diff>